<commit_message>
Support optional third CTF pole
</commit_message>
<xml_diff>
--- a/cases/c2m_8023dj_4p13p0_50mm/config/config_178A.xlsx
+++ b/cases/c2m_8023dj_4p13p0_50mm/config/config_178A.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="fixed_config" sheetId="1" r:id="R85058fe0fdd7419f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="search_config" sheetId="2" r:id="Re12f6da248e24df3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="channels" sheetId="3" r:id="R1859a41724eb4ac3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="run_config" sheetId="4" r:id="R7535a131be214173"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="fixed_config" sheetId="1" r:id="Re863ed1c0bc64969"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="search_config" sheetId="2" r:id="Rd4f6cc0ea54544bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="channels" sheetId="3" r:id="R20d56dfb68014d30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="run_config" sheetId="4" r:id="R687cd566bf204a30"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -193,9 +193,6 @@
     <x:t xml:space="preserve">f_p3</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">178A CTF pole 3; explicit project setting at f_b.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">A_v</x:t>
   </x:si>
   <x:si>
@@ -977,26 +974,115 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Profile</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">single_run</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">target</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">dfe</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Full single-run target.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">pre_dte_pmf_method</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Pre-DTE ADC PMF method for V_qc.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">pmf_grid_quality</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">coarse</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">PMF amplitude-grid quality.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">floating_mode</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">simplified</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">FFE floating-group selection.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">pos_sweep_method</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">each_phase</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Sampling-phase sweep strategy.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">pos_coarse_stride</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">phase index</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Coarse phase stride; used only by coarse_fine.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">search_sweep</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">mse</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Partial-search candidate evaluation target.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">heuristic</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">coarse_fine</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">search_final</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Top-K final evaluation target.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">fine</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">search</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">group_size</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Manifest candidates per partial-search group.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">top_k</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Minimum-MSE candidates re-evaluated by search_final.</x:t>
   </x:si>
 </x:sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="11">
+  <x:numFmts count="7">
     <x:numFmt numFmtId="164" formatCode="General"/>
     <x:numFmt numFmtId="165" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* \-??_-;_-@_-"/>
-    <x:numFmt numFmtId="166" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* \-??_-;_-@_-"/>
-    <x:numFmt numFmtId="167" formatCode="_-* #,##0_-;\-* #,##0_-;_-* \-_-;_-@_-"/>
-    <x:numFmt numFmtId="168" formatCode="_-* #,##0_-;\-* #,##0_-;_-* \-_-;_-@_-"/>
-    <x:numFmt numFmtId="169" formatCode="_-\$* #,##0.00_-;&quot;-$&quot;* #,##0.00_-;_-\$* \-??_-;_-@_-"/>
-    <x:numFmt numFmtId="170" formatCode="_-\$* #,##0.00_-;&quot;-$&quot;* #,##0.00_-;_-\$* \-??_-;_-@_-"/>
-    <x:numFmt numFmtId="171" formatCode="_-\$* #,##0_-;&quot;-$&quot;* #,##0_-;_-\$* \-_-;_-@_-"/>
-    <x:numFmt numFmtId="172" formatCode="_-\$* #,##0_-;&quot;-$&quot;* #,##0_-;_-\$* \-_-;_-@_-"/>
-    <x:numFmt numFmtId="173" formatCode="0%"/>
-    <x:numFmt numFmtId="174" formatCode="0.000000E+00"/>
+    <x:numFmt numFmtId="166" formatCode="_-* #,##0_-;\-* #,##0_-;_-* \-_-;_-@_-"/>
+    <x:numFmt numFmtId="167" formatCode="_-\$* #,##0.00_-;&quot;-$&quot;* #,##0.00_-;_-\$* \-??_-;_-@_-"/>
+    <x:numFmt numFmtId="168" formatCode="_-\$* #,##0_-;&quot;-$&quot;* #,##0_-;_-\$* \-_-;_-@_-"/>
+    <x:numFmt numFmtId="169" formatCode="0%"/>
+    <x:numFmt numFmtId="170" formatCode="0.000000E+00"/>
   </x:numFmts>
-  <x:fonts count="9">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="10"/>
       <x:name val="Noto Sans TC"/>
@@ -1037,6 +1123,10 @@
       <x:color rgb="FF1F1F1F"/>
       <x:name val="Calibri"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
   <x:fills count="4">
     <x:fill>
@@ -1073,7 +1163,7 @@
       </x:bottom>
     </x:border>
   </x:borders>
-  <x:cellStyleXfs count="33">
+  <x:cellStyleXfs count="39">
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0"/>
       <x:protection locked="1" hidden="0"/>
@@ -1097,20 +1187,40 @@
     <x:xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <x:xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <x:xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <x:xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <x:xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0"/>
+    </x:xf>
     <x:xf numFmtId="166" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="0">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0"/>
     </x:xf>
-    <x:xf numFmtId="167" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <x:xf numFmtId="166" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0"/>
+    </x:xf>
+    <x:xf numFmtId="166" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0"/>
+    </x:xf>
+    <x:xf numFmtId="167" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0"/>
+    </x:xf>
+    <x:xf numFmtId="167" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0"/>
+    </x:xf>
+    <x:xf numFmtId="167" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0"/>
+    </x:xf>
     <x:xf numFmtId="168" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="0">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0"/>
     </x:xf>
-    <x:xf numFmtId="169" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <x:xf numFmtId="170" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <x:xf numFmtId="168" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="0">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0"/>
     </x:xf>
-    <x:xf numFmtId="171" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <x:xf numFmtId="172" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <x:xf numFmtId="168" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="0">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0"/>
     </x:xf>
     <x:xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1125,38 +1235,56 @@
       <x:alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="173" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <x:xf numFmtId="173" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <x:xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="169" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0"/>
+    </x:xf>
+    <x:xf numFmtId="169" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0"/>
+    </x:xf>
+    <x:xf numFmtId="169" fontId="4" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="1" applyProtection="0">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="8">
+  <x:cellXfs count="11">
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="0" applyBorder="0" applyAlignment="0">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
     </x:xf>
-    <x:xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="28" applyFont="0" applyBorder="0" applyAlignment="1">
+    <x:xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="35" applyFont="0" applyBorder="0" applyAlignment="1">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
     </x:xf>
-    <x:xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="29" applyFont="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="33" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="bottom" wrapText="0"/>
     </x:xf>
-    <x:xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="29" applyFont="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="33" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="0"/>
     </x:xf>
-    <x:xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="29" applyFont="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="33" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="general" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="174" fontId="6" fillId="0" borderId="1" xfId="29" applyFont="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="170" fontId="6" fillId="0" borderId="1" xfId="33" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="general" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="28" applyFont="1" applyBorder="0" applyAlignment="1">
+    <x:xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="35" applyFont="1" applyBorder="0" applyAlignment="1">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
     </x:xf>
-    <x:xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="28" applyFont="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="0" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="35" applyFont="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="35" applyFont="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="0" applyAlignment="1">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
-  <x:cellStyles count="19">
+  <x:cellStyles count="25">
     <x:cellStyle name="Normal" xfId="0"/>
     <x:cellStyle name="Comma" xfId="15"/>
     <x:cellStyle name="Comma [0]" xfId="16"/>
@@ -1165,17 +1293,23 @@
     <x:cellStyle name="Percent" xfId="19"/>
     <x:cellStyle name="Comma" xfId="20"/>
     <x:cellStyle name="Comma 1" xfId="21"/>
-    <x:cellStyle name="Comma [0]" xfId="22"/>
-    <x:cellStyle name="Comma [0] 2" xfId="23"/>
-    <x:cellStyle name="Currency" xfId="24"/>
-    <x:cellStyle name="Currency 3" xfId="25"/>
-    <x:cellStyle name="Currency [0]" xfId="26"/>
-    <x:cellStyle name="Currency [0] 4" xfId="27"/>
-    <x:cellStyle name="Normal" xfId="28"/>
-    <x:cellStyle name="Normal 1" xfId="29"/>
-    <x:cellStyle name="Normal 5" xfId="30"/>
-    <x:cellStyle name="Percent" xfId="31"/>
-    <x:cellStyle name="Percent 6" xfId="32"/>
+    <x:cellStyle name="Comma 2" xfId="22"/>
+    <x:cellStyle name="Comma [0]" xfId="23"/>
+    <x:cellStyle name="Comma [0] 2" xfId="24"/>
+    <x:cellStyle name="Comma [0] 3" xfId="25"/>
+    <x:cellStyle name="Currency" xfId="26"/>
+    <x:cellStyle name="Currency 3" xfId="27"/>
+    <x:cellStyle name="Currency 4" xfId="28"/>
+    <x:cellStyle name="Currency [0]" xfId="29"/>
+    <x:cellStyle name="Currency [0] 4" xfId="30"/>
+    <x:cellStyle name="Currency [0] 5" xfId="31"/>
+    <x:cellStyle name="Normal" xfId="32"/>
+    <x:cellStyle name="Normal 1" xfId="33"/>
+    <x:cellStyle name="Normal 5" xfId="34"/>
+    <x:cellStyle name="Normal 6" xfId="35"/>
+    <x:cellStyle name="Percent" xfId="36"/>
+    <x:cellStyle name="Percent 6" xfId="37"/>
+    <x:cellStyle name="Percent 7" xfId="38"/>
   </x:cellStyles>
   <x:colors>
     <x:indexedColors>
@@ -1792,14 +1926,12 @@
       <x:c r="B24" s="4" t="s">
         <x:v>59</x:v>
       </x:c>
-      <x:c r="C24" s="5" t="n">
-        <x:v>106250000000</x:v>
-      </x:c>
+      <x:c r="C24" s="5"/>
       <x:c r="D24" s="4" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="E24" s="4" t="s">
-        <x:v>60</x:v>
+      <x:c r="E24" s="4" t="str">
+        <x:v>Optional 178A CTF pole 3; leave blank to bypass the third pole.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0">
@@ -1807,16 +1939,16 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="B25" s="4" t="s">
-        <x:v>61</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C25" s="5" t="n">
         <x:v>0.385</x:v>
       </x:c>
       <x:c r="D25" s="4" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="E25" s="4" t="s">
         <x:v>62</x:v>
-      </x:c>
-      <x:c r="E25" s="4" t="s">
-        <x:v>63</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15" hidden="0">
@@ -1824,16 +1956,16 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="B26" s="4" t="s">
-        <x:v>64</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="C26" s="5" t="n">
         <x:v>0.385</x:v>
       </x:c>
       <x:c r="D26" s="4" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="E26" s="4" t="s">
-        <x:v>65</x:v>
+        <x:v>64</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15" hidden="0">
@@ -1841,1388 +1973,1388 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="B27" s="4" t="s">
-        <x:v>66</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="C27" s="5" t="n">
         <x:v>0.481</x:v>
       </x:c>
       <x:c r="D27" s="4" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="E27" s="4" t="s">
-        <x:v>67</x:v>
+        <x:v>66</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="15" hidden="0">
       <x:c r="A28" s="4" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="B28" s="4" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="B28" s="4" t="s">
+      <x:c r="C28" s="5" t="s">
         <x:v>69</x:v>
       </x:c>
-      <x:c r="C28" s="5" t="s">
+      <x:c r="D28" s="4" t="s">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="D28" s="4" t="s">
+      <x:c r="E28" s="4" t="s">
         <x:v>71</x:v>
-      </x:c>
-      <x:c r="E28" s="4" t="s">
-        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15" hidden="0">
       <x:c r="A29" s="4" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B29" s="4" t="s">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="C29" s="5" t="s">
         <x:v>73</x:v>
       </x:c>
-      <x:c r="C29" s="5" t="s">
+      <x:c r="D29" s="4" t="s">
         <x:v>74</x:v>
       </x:c>
-      <x:c r="D29" s="4" t="s">
+      <x:c r="E29" s="4" t="s">
         <x:v>75</x:v>
-      </x:c>
-      <x:c r="E29" s="4" t="s">
-        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15" hidden="0">
       <x:c r="A30" s="4" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B30" s="4" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C30" s="5" t="n">
         <x:v>3E-014</x:v>
       </x:c>
       <x:c r="D30" s="4" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E30" s="4" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="15" hidden="0">
       <x:c r="A31" s="4" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B31" s="4" t="s">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="C31" s="5" t="s">
         <x:v>79</x:v>
       </x:c>
-      <x:c r="C31" s="5" t="s">
+      <x:c r="D31" s="4" t="s">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="D31" s="4" t="s">
+      <x:c r="E31" s="4" t="s">
         <x:v>81</x:v>
-      </x:c>
-      <x:c r="E31" s="4" t="s">
-        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="15" hidden="0">
       <x:c r="A32" s="4" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B32" s="4" t="s">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="C32" s="5" t="s">
         <x:v>83</x:v>
       </x:c>
-      <x:c r="C32" s="5" t="s">
+      <x:c r="D32" s="4" t="s">
         <x:v>84</x:v>
       </x:c>
-      <x:c r="D32" s="4" t="s">
+      <x:c r="E32" s="4" t="s">
         <x:v>85</x:v>
-      </x:c>
-      <x:c r="E32" s="4" t="s">
-        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15" hidden="0">
       <x:c r="A33" s="4" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B33" s="4" t="s">
-        <x:v>87</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="C33" s="5" t="n">
         <x:v>0.0005</x:v>
       </x:c>
       <x:c r="D33" s="4" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="E33" s="4" t="s">
         <x:v>88</x:v>
-      </x:c>
-      <x:c r="E33" s="4" t="s">
-        <x:v>89</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15" hidden="0">
       <x:c r="A34" s="4" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B34" s="4" t="s">
-        <x:v>90</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="C34" s="5" t="n">
         <x:v>0.00065</x:v>
       </x:c>
       <x:c r="D34" s="4" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="E34" s="4" t="s">
         <x:v>91</x:v>
-      </x:c>
-      <x:c r="E34" s="4" t="s">
-        <x:v>92</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="15" hidden="0">
       <x:c r="A35" s="4" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B35" s="4" t="s">
-        <x:v>93</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="C35" s="5" t="n">
         <x:v>0.000293</x:v>
       </x:c>
       <x:c r="D35" s="4" t="s">
-        <x:v>91</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="E35" s="4" t="s">
-        <x:v>94</x:v>
+        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15" hidden="0">
       <x:c r="A36" s="4" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B36" s="4" t="s">
-        <x:v>95</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="C36" s="5" t="n">
         <x:v>0.006141</x:v>
       </x:c>
       <x:c r="D36" s="4" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="E36" s="4" t="s">
         <x:v>96</x:v>
-      </x:c>
-      <x:c r="E36" s="4" t="s">
-        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15" hidden="0">
       <x:c r="A37" s="4" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B37" s="4" t="s">
-        <x:v>98</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="C37" s="5" t="n">
         <x:v>4E-014</x:v>
       </x:c>
       <x:c r="D37" s="4" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E37" s="4" t="s">
-        <x:v>99</x:v>
+        <x:v>98</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="15" hidden="0">
       <x:c r="A38" s="4" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B38" s="4" t="s">
-        <x:v>100</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="C38" s="5" t="b">
         <x:f aca="0">FALSE()</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D38" s="4" t="s">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E38" s="4" t="s">
         <x:v>101</x:v>
-      </x:c>
-      <x:c r="E38" s="4" t="s">
-        <x:v>102</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="15" hidden="0">
       <x:c r="A39" s="4" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B39" s="4" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="C39" s="5" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D39" s="4" t="s">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="E39" s="4" t="s">
         <x:v>103</x:v>
-      </x:c>
-      <x:c r="C39" s="5" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D39" s="4" t="s">
-        <x:v>71</x:v>
-      </x:c>
-      <x:c r="E39" s="4" t="s">
-        <x:v>104</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15" hidden="0">
       <x:c r="A40" s="4" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B40" s="4" t="s">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="C40" s="5" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D40" s="4" t="s">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="E40" s="4" t="s">
         <x:v>105</x:v>
-      </x:c>
-      <x:c r="C40" s="5" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D40" s="4" t="s">
-        <x:v>71</x:v>
-      </x:c>
-      <x:c r="E40" s="4" t="s">
-        <x:v>106</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="15" hidden="0">
       <x:c r="A41" s="4" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B41" s="4" t="s">
-        <x:v>107</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="C41" s="5" t="n">
         <x:v>9</x:v>
       </x:c>
       <x:c r="D41" s="4" t="s">
-        <x:v>81</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="E41" s="4" t="s">
-        <x:v>108</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="15" hidden="0">
       <x:c r="A42" s="4" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B42" s="4" t="s">
-        <x:v>109</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="C42" s="5" t="n">
         <x:v>92.5</x:v>
       </x:c>
       <x:c r="D42" s="4" t="s">
-        <x:v>85</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="E42" s="4" t="s">
-        <x:v>110</x:v>
+        <x:v>109</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="15" hidden="0">
       <x:c r="A43" s="4" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B43" s="4" t="s">
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="C43" s="5" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D43" s="4" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="E43" s="4" t="s">
         <x:v>111</x:v>
-      </x:c>
-      <x:c r="C43" s="5" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D43" s="4" t="s">
-        <x:v>88</x:v>
-      </x:c>
-      <x:c r="E43" s="4" t="s">
-        <x:v>112</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="15" hidden="0">
       <x:c r="A44" s="4" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B44" s="4" t="s">
-        <x:v>113</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="C44" s="5" t="n">
         <x:v>0.000595</x:v>
       </x:c>
       <x:c r="D44" s="4" t="s">
+        <x:v>113</x:v>
+      </x:c>
+      <x:c r="E44" s="4" t="s">
         <x:v>114</x:v>
-      </x:c>
-      <x:c r="E44" s="4" t="s">
-        <x:v>115</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="15" hidden="0">
       <x:c r="A45" s="4" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B45" s="4" t="s">
-        <x:v>116</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="C45" s="5" t="n">
         <x:v>2.6E-005</x:v>
       </x:c>
       <x:c r="D45" s="4" t="s">
-        <x:v>114</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="E45" s="4" t="s">
-        <x:v>117</x:v>
+        <x:v>116</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="15" hidden="0">
       <x:c r="A46" s="4" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B46" s="4" t="s">
-        <x:v>118</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="C46" s="5" t="n">
         <x:v>0.00579</x:v>
       </x:c>
       <x:c r="D46" s="4" t="s">
-        <x:v>96</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="E46" s="4" t="s">
-        <x:v>119</x:v>
+        <x:v>118</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="15" hidden="0">
       <x:c r="A47" s="4" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B47" s="4" t="s">
-        <x:v>120</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="C47" s="5" t="n">
         <x:v>46.25</x:v>
       </x:c>
       <x:c r="D47" s="4" t="s">
-        <x:v>85</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="E47" s="4" t="s">
-        <x:v>121</x:v>
+        <x:v>120</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="15" hidden="0">
       <x:c r="A48" s="4" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="B48" s="4" t="s">
         <x:v>122</x:v>
       </x:c>
-      <x:c r="B48" s="4" t="s">
-        <x:v>123</x:v>
-      </x:c>
       <x:c r="C48" s="5" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="D48" s="4" t="s">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="D48" s="4" t="s">
+      <x:c r="E48" s="4" t="s">
         <x:v>71</x:v>
-      </x:c>
-      <x:c r="E48" s="4" t="s">
-        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="15" hidden="0">
       <x:c r="A49" s="4" t="s">
-        <x:v>122</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B49" s="4" t="s">
-        <x:v>124</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="C49" s="5" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="D49" s="4" t="s">
         <x:v>74</x:v>
       </x:c>
-      <x:c r="D49" s="4" t="s">
+      <x:c r="E49" s="4" t="s">
         <x:v>75</x:v>
-      </x:c>
-      <x:c r="E49" s="4" t="s">
-        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0">
       <x:c r="A50" s="4" t="s">
-        <x:v>122</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B50" s="4" t="s">
-        <x:v>125</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="C50" s="5" t="n">
         <x:v>3E-014</x:v>
       </x:c>
       <x:c r="D50" s="4" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E50" s="4" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="15" hidden="0">
       <x:c r="A51" s="4" t="s">
-        <x:v>122</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B51" s="4" t="s">
-        <x:v>126</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="C51" s="5" t="s">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="D51" s="4" t="s">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="D51" s="4" t="s">
+      <x:c r="E51" s="4" t="s">
         <x:v>81</x:v>
-      </x:c>
-      <x:c r="E51" s="4" t="s">
-        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="15" hidden="0">
       <x:c r="A52" s="4" t="s">
-        <x:v>122</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B52" s="4" t="s">
-        <x:v>127</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="C52" s="5" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="D52" s="4" t="s">
         <x:v>84</x:v>
       </x:c>
-      <x:c r="D52" s="4" t="s">
+      <x:c r="E52" s="4" t="s">
         <x:v>85</x:v>
-      </x:c>
-      <x:c r="E52" s="4" t="s">
-        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="15" hidden="0">
       <x:c r="A53" s="4" t="s">
-        <x:v>122</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B53" s="4" t="s">
-        <x:v>128</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="C53" s="5" t="n">
         <x:v>0.0005</x:v>
       </x:c>
       <x:c r="D53" s="4" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="E53" s="4" t="s">
         <x:v>88</x:v>
-      </x:c>
-      <x:c r="E53" s="4" t="s">
-        <x:v>89</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="15" hidden="0">
       <x:c r="A54" s="4" t="s">
-        <x:v>122</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B54" s="4" t="s">
-        <x:v>129</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="C54" s="5" t="n">
         <x:v>0.00065</x:v>
       </x:c>
       <x:c r="D54" s="4" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="E54" s="4" t="s">
         <x:v>91</x:v>
-      </x:c>
-      <x:c r="E54" s="4" t="s">
-        <x:v>92</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="15" hidden="0">
       <x:c r="A55" s="4" t="s">
-        <x:v>122</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B55" s="4" t="s">
-        <x:v>130</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="C55" s="5" t="n">
         <x:v>0.000293</x:v>
       </x:c>
       <x:c r="D55" s="4" t="s">
-        <x:v>91</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="E55" s="4" t="s">
-        <x:v>94</x:v>
+        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="15" hidden="0">
       <x:c r="A56" s="4" t="s">
-        <x:v>122</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B56" s="4" t="s">
-        <x:v>131</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="C56" s="5" t="n">
         <x:v>0.006141</x:v>
       </x:c>
       <x:c r="D56" s="4" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="E56" s="4" t="s">
         <x:v>96</x:v>
-      </x:c>
-      <x:c r="E56" s="4" t="s">
-        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="15" hidden="0">
       <x:c r="A57" s="4" t="s">
-        <x:v>122</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B57" s="4" t="s">
-        <x:v>132</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="C57" s="5" t="n">
         <x:v>4E-014</x:v>
       </x:c>
       <x:c r="D57" s="4" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E57" s="4" t="s">
-        <x:v>99</x:v>
+        <x:v>98</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="15" hidden="0">
       <x:c r="A58" s="4" t="s">
-        <x:v>122</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B58" s="4" t="s">
-        <x:v>133</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="C58" s="5" t="b">
         <x:f aca="0">FALSE()</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D58" s="4" t="s">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E58" s="4" t="s">
         <x:v>101</x:v>
-      </x:c>
-      <x:c r="E58" s="4" t="s">
-        <x:v>102</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="15" hidden="0">
       <x:c r="A59" s="4" t="s">
-        <x:v>122</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B59" s="4" t="s">
-        <x:v>134</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="C59" s="5" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D59" s="4" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E59" s="4" t="s">
-        <x:v>104</x:v>
+        <x:v>103</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="15" hidden="0">
       <x:c r="A60" s="4" t="s">
-        <x:v>122</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B60" s="4" t="s">
-        <x:v>135</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="C60" s="5" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D60" s="4" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E60" s="4" t="s">
-        <x:v>106</x:v>
+        <x:v>105</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="15" hidden="0">
       <x:c r="A61" s="4" t="s">
-        <x:v>122</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B61" s="4" t="s">
-        <x:v>136</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="C61" s="5" t="n">
         <x:v>9</x:v>
       </x:c>
       <x:c r="D61" s="4" t="s">
-        <x:v>81</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="E61" s="4" t="s">
-        <x:v>108</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="15" hidden="0">
       <x:c r="A62" s="4" t="s">
-        <x:v>122</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B62" s="4" t="s">
-        <x:v>137</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="C62" s="5" t="n">
         <x:v>92.5</x:v>
       </x:c>
       <x:c r="D62" s="4" t="s">
-        <x:v>85</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="E62" s="4" t="s">
-        <x:v>110</x:v>
+        <x:v>109</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="15" hidden="0">
       <x:c r="A63" s="4" t="s">
-        <x:v>122</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B63" s="4" t="s">
-        <x:v>138</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="C63" s="5" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D63" s="4" t="s">
-        <x:v>88</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="E63" s="4" t="s">
-        <x:v>112</x:v>
+        <x:v>111</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="15" hidden="0">
       <x:c r="A64" s="4" t="s">
-        <x:v>122</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B64" s="4" t="s">
-        <x:v>139</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="C64" s="5" t="n">
         <x:v>0.000595</x:v>
       </x:c>
       <x:c r="D64" s="4" t="s">
+        <x:v>113</x:v>
+      </x:c>
+      <x:c r="E64" s="4" t="s">
         <x:v>114</x:v>
-      </x:c>
-      <x:c r="E64" s="4" t="s">
-        <x:v>115</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="15" hidden="0">
       <x:c r="A65" s="4" t="s">
-        <x:v>122</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B65" s="4" t="s">
-        <x:v>140</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="C65" s="5" t="n">
         <x:v>2.6E-005</x:v>
       </x:c>
       <x:c r="D65" s="4" t="s">
-        <x:v>114</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="E65" s="4" t="s">
-        <x:v>117</x:v>
+        <x:v>116</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="15" hidden="0">
       <x:c r="A66" s="4" t="s">
-        <x:v>122</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B66" s="4" t="s">
-        <x:v>141</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="C66" s="5" t="n">
         <x:v>0.00579</x:v>
       </x:c>
       <x:c r="D66" s="4" t="s">
-        <x:v>96</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="E66" s="4" t="s">
-        <x:v>119</x:v>
+        <x:v>118</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="15" hidden="0">
       <x:c r="A67" s="4" t="s">
-        <x:v>122</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B67" s="4" t="s">
-        <x:v>142</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="C67" s="5" t="n">
         <x:v>46.25</x:v>
       </x:c>
       <x:c r="D67" s="4" t="s">
-        <x:v>85</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="E67" s="4" t="s">
-        <x:v>121</x:v>
+        <x:v>120</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="15" hidden="0">
       <x:c r="A68" s="4" t="s">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="B68" s="4" t="s">
         <x:v>143</x:v>
       </x:c>
-      <x:c r="B68" s="4" t="s">
-        <x:v>144</x:v>
-      </x:c>
       <x:c r="C68" s="5" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="D68" s="4" t="s">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="D68" s="4" t="s">
+      <x:c r="E68" s="4" t="s">
         <x:v>71</x:v>
-      </x:c>
-      <x:c r="E68" s="4" t="s">
-        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="15" hidden="0">
       <x:c r="A69" s="4" t="s">
-        <x:v>143</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B69" s="4" t="s">
-        <x:v>145</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="C69" s="5" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="D69" s="4" t="s">
         <x:v>74</x:v>
       </x:c>
-      <x:c r="D69" s="4" t="s">
+      <x:c r="E69" s="4" t="s">
         <x:v>75</x:v>
-      </x:c>
-      <x:c r="E69" s="4" t="s">
-        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="15" hidden="0">
       <x:c r="A70" s="4" t="s">
-        <x:v>143</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B70" s="4" t="s">
-        <x:v>146</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="C70" s="5" t="n">
         <x:v>3E-014</x:v>
       </x:c>
       <x:c r="D70" s="4" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E70" s="4" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="15" hidden="0">
       <x:c r="A71" s="4" t="s">
-        <x:v>143</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B71" s="4" t="s">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="C71" s="5" t="s">
         <x:v>147</x:v>
       </x:c>
-      <x:c r="C71" s="5" t="s">
-        <x:v>148</x:v>
-      </x:c>
       <x:c r="D71" s="4" t="s">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="E71" s="4" t="s">
         <x:v>81</x:v>
-      </x:c>
-      <x:c r="E71" s="4" t="s">
-        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="15" hidden="0">
       <x:c r="A72" s="4" t="s">
-        <x:v>143</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B72" s="4" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="C72" s="5" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="D72" s="4" t="s">
         <x:v>84</x:v>
       </x:c>
-      <x:c r="D72" s="4" t="s">
+      <x:c r="E72" s="4" t="s">
         <x:v>85</x:v>
-      </x:c>
-      <x:c r="E72" s="4" t="s">
-        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="15" hidden="0">
       <x:c r="A73" s="4" t="s">
-        <x:v>143</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B73" s="4" t="s">
-        <x:v>150</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="C73" s="5" t="n">
         <x:v>0.0005</x:v>
       </x:c>
       <x:c r="D73" s="4" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="E73" s="4" t="s">
         <x:v>88</x:v>
-      </x:c>
-      <x:c r="E73" s="4" t="s">
-        <x:v>89</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="15" hidden="0">
       <x:c r="A74" s="4" t="s">
-        <x:v>143</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B74" s="4" t="s">
-        <x:v>151</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="C74" s="5" t="n">
         <x:v>0.00065</x:v>
       </x:c>
       <x:c r="D74" s="4" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="E74" s="4" t="s">
         <x:v>91</x:v>
-      </x:c>
-      <x:c r="E74" s="4" t="s">
-        <x:v>92</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="15" hidden="0">
       <x:c r="A75" s="4" t="s">
-        <x:v>143</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B75" s="4" t="s">
-        <x:v>152</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="C75" s="5" t="n">
         <x:v>0.000293</x:v>
       </x:c>
       <x:c r="D75" s="4" t="s">
-        <x:v>91</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="E75" s="4" t="s">
-        <x:v>94</x:v>
+        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="15" hidden="0">
       <x:c r="A76" s="4" t="s">
-        <x:v>143</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B76" s="4" t="s">
-        <x:v>153</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="C76" s="5" t="n">
         <x:v>0.006141</x:v>
       </x:c>
       <x:c r="D76" s="4" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="E76" s="4" t="s">
         <x:v>96</x:v>
-      </x:c>
-      <x:c r="E76" s="4" t="s">
-        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="15" hidden="0">
       <x:c r="A77" s="4" t="s">
-        <x:v>143</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B77" s="4" t="s">
-        <x:v>154</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C77" s="5" t="n">
         <x:v>4E-014</x:v>
       </x:c>
       <x:c r="D77" s="4" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E77" s="4" t="s">
-        <x:v>99</x:v>
+        <x:v>98</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="15" hidden="0">
       <x:c r="A78" s="4" t="s">
-        <x:v>143</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B78" s="4" t="s">
-        <x:v>155</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="C78" s="5" t="b">
         <x:f aca="0">FALSE()</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D78" s="4" t="s">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E78" s="4" t="s">
         <x:v>101</x:v>
-      </x:c>
-      <x:c r="E78" s="4" t="s">
-        <x:v>102</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="15" hidden="0">
       <x:c r="A79" s="4" t="s">
-        <x:v>143</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B79" s="4" t="s">
-        <x:v>156</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="C79" s="5" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D79" s="4" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E79" s="4" t="s">
-        <x:v>104</x:v>
+        <x:v>103</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="15" hidden="0">
       <x:c r="A80" s="4" t="s">
-        <x:v>143</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B80" s="4" t="s">
-        <x:v>157</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="C80" s="5" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D80" s="4" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E80" s="4" t="s">
-        <x:v>106</x:v>
+        <x:v>105</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="15" hidden="0">
       <x:c r="A81" s="4" t="s">
-        <x:v>143</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B81" s="4" t="s">
-        <x:v>158</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="C81" s="5" t="n">
         <x:v>9</x:v>
       </x:c>
       <x:c r="D81" s="4" t="s">
-        <x:v>81</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="E81" s="4" t="s">
-        <x:v>108</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="15" hidden="0">
       <x:c r="A82" s="4" t="s">
-        <x:v>143</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B82" s="4" t="s">
-        <x:v>159</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="C82" s="5" t="n">
         <x:v>92.5</x:v>
       </x:c>
       <x:c r="D82" s="4" t="s">
-        <x:v>85</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="E82" s="4" t="s">
-        <x:v>110</x:v>
+        <x:v>109</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="15" hidden="0">
       <x:c r="A83" s="4" t="s">
-        <x:v>143</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B83" s="4" t="s">
-        <x:v>160</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="C83" s="5" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D83" s="4" t="s">
-        <x:v>88</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="E83" s="4" t="s">
-        <x:v>112</x:v>
+        <x:v>111</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="15" hidden="0">
       <x:c r="A84" s="4" t="s">
-        <x:v>143</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B84" s="4" t="s">
-        <x:v>161</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="C84" s="5" t="n">
         <x:v>0.000595</x:v>
       </x:c>
       <x:c r="D84" s="4" t="s">
+        <x:v>113</x:v>
+      </x:c>
+      <x:c r="E84" s="4" t="s">
         <x:v>114</x:v>
-      </x:c>
-      <x:c r="E84" s="4" t="s">
-        <x:v>115</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="15" hidden="0">
       <x:c r="A85" s="4" t="s">
-        <x:v>143</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B85" s="4" t="s">
-        <x:v>162</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="C85" s="5" t="n">
         <x:v>2.6E-005</x:v>
       </x:c>
       <x:c r="D85" s="4" t="s">
-        <x:v>114</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="E85" s="4" t="s">
-        <x:v>117</x:v>
+        <x:v>116</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="15" hidden="0">
       <x:c r="A86" s="4" t="s">
-        <x:v>143</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B86" s="4" t="s">
-        <x:v>163</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="C86" s="5" t="n">
         <x:v>0.00579</x:v>
       </x:c>
       <x:c r="D86" s="4" t="s">
-        <x:v>96</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="E86" s="4" t="s">
-        <x:v>119</x:v>
+        <x:v>118</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="15" hidden="0">
       <x:c r="A87" s="4" t="s">
-        <x:v>143</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B87" s="4" t="s">
-        <x:v>164</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="C87" s="5" t="n">
         <x:v>46.25</x:v>
       </x:c>
       <x:c r="D87" s="4" t="s">
-        <x:v>85</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="E87" s="4" t="s">
-        <x:v>121</x:v>
+        <x:v>120</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="15" hidden="0">
       <x:c r="A88" s="4" t="s">
+        <x:v>164</x:v>
+      </x:c>
+      <x:c r="B88" s="4" t="s">
         <x:v>165</x:v>
       </x:c>
-      <x:c r="B88" s="4" t="s">
-        <x:v>166</x:v>
-      </x:c>
       <x:c r="C88" s="5" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="D88" s="4" t="s">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="D88" s="4" t="s">
+      <x:c r="E88" s="4" t="s">
         <x:v>71</x:v>
-      </x:c>
-      <x:c r="E88" s="4" t="s">
-        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="15" hidden="0">
       <x:c r="A89" s="4" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B89" s="4" t="s">
-        <x:v>167</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="C89" s="5" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="D89" s="4" t="s">
         <x:v>74</x:v>
       </x:c>
-      <x:c r="D89" s="4" t="s">
+      <x:c r="E89" s="4" t="s">
         <x:v>75</x:v>
-      </x:c>
-      <x:c r="E89" s="4" t="s">
-        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="15" hidden="0">
       <x:c r="A90" s="4" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B90" s="4" t="s">
-        <x:v>168</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="C90" s="5" t="n">
         <x:v>3E-014</x:v>
       </x:c>
       <x:c r="D90" s="4" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E90" s="4" t="s">
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="15" hidden="0">
       <x:c r="A91" s="4" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B91" s="4" t="s">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="C91" s="5" t="s">
         <x:v>169</x:v>
       </x:c>
-      <x:c r="C91" s="5" t="s">
-        <x:v>170</x:v>
-      </x:c>
       <x:c r="D91" s="4" t="s">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="E91" s="4" t="s">
         <x:v>81</x:v>
-      </x:c>
-      <x:c r="E91" s="4" t="s">
-        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="15" hidden="0">
       <x:c r="A92" s="4" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B92" s="4" t="s">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="C92" s="5" t="s">
         <x:v>171</x:v>
       </x:c>
-      <x:c r="C92" s="5" t="s">
-        <x:v>172</x:v>
-      </x:c>
       <x:c r="D92" s="4" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="E92" s="4" t="s">
         <x:v>85</x:v>
-      </x:c>
-      <x:c r="E92" s="4" t="s">
-        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="15" hidden="0">
       <x:c r="A93" s="4" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B93" s="4" t="s">
-        <x:v>173</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="C93" s="5" t="n">
         <x:v>0.0005</x:v>
       </x:c>
       <x:c r="D93" s="4" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="E93" s="4" t="s">
         <x:v>88</x:v>
-      </x:c>
-      <x:c r="E93" s="4" t="s">
-        <x:v>89</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="15" hidden="0">
       <x:c r="A94" s="4" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B94" s="4" t="s">
-        <x:v>174</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="C94" s="5" t="n">
         <x:v>0.00089</x:v>
       </x:c>
       <x:c r="D94" s="4" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="E94" s="4" t="s">
         <x:v>91</x:v>
-      </x:c>
-      <x:c r="E94" s="4" t="s">
-        <x:v>92</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="15" hidden="0">
       <x:c r="A95" s="4" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B95" s="4" t="s">
-        <x:v>175</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="C95" s="5" t="n">
         <x:v>0.0002</x:v>
       </x:c>
       <x:c r="D95" s="4" t="s">
-        <x:v>91</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="E95" s="4" t="s">
-        <x:v>94</x:v>
+        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="15" hidden="0">
       <x:c r="A96" s="4" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B96" s="4" t="s">
-        <x:v>176</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="C96" s="5" t="n">
         <x:v>0.006141</x:v>
       </x:c>
       <x:c r="D96" s="4" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="E96" s="4" t="s">
         <x:v>96</x:v>
-      </x:c>
-      <x:c r="E96" s="4" t="s">
-        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="15" hidden="0">
       <x:c r="A97" s="4" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B97" s="4" t="s">
-        <x:v>177</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="C97" s="5" t="n">
         <x:v>4E-014</x:v>
       </x:c>
       <x:c r="D97" s="4" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E97" s="4" t="s">
-        <x:v>99</x:v>
+        <x:v>98</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="15" hidden="0">
       <x:c r="A98" s="4" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B98" s="4" t="s">
-        <x:v>178</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="C98" s="5" t="b">
         <x:f aca="0">FALSE()</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D98" s="4" t="s">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E98" s="4" t="s">
         <x:v>101</x:v>
-      </x:c>
-      <x:c r="E98" s="4" t="s">
-        <x:v>102</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="15" hidden="0">
       <x:c r="A99" s="4" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B99" s="4" t="s">
-        <x:v>179</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="C99" s="5" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D99" s="4" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E99" s="4" t="s">
-        <x:v>104</x:v>
+        <x:v>103</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="15" hidden="0">
       <x:c r="A100" s="4" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B100" s="4" t="s">
-        <x:v>180</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="C100" s="5" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D100" s="4" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E100" s="4" t="s">
-        <x:v>106</x:v>
+        <x:v>105</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="15" hidden="0">
       <x:c r="A101" s="4" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B101" s="4" t="s">
-        <x:v>181</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="C101" s="5" t="n">
         <x:v>9</x:v>
       </x:c>
       <x:c r="D101" s="4" t="s">
-        <x:v>81</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="E101" s="4" t="s">
-        <x:v>108</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="15" hidden="0">
       <x:c r="A102" s="4" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B102" s="4" t="s">
-        <x:v>182</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="C102" s="5" t="n">
         <x:v>92.5</x:v>
       </x:c>
       <x:c r="D102" s="4" t="s">
-        <x:v>85</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="E102" s="4" t="s">
-        <x:v>110</x:v>
+        <x:v>109</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="15" hidden="0">
       <x:c r="A103" s="4" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B103" s="4" t="s">
-        <x:v>183</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="C103" s="5" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D103" s="4" t="s">
-        <x:v>88</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="E103" s="4" t="s">
-        <x:v>112</x:v>
+        <x:v>111</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="15" hidden="0">
       <x:c r="A104" s="4" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B104" s="4" t="s">
-        <x:v>184</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="C104" s="5" t="n">
         <x:v>0.000595</x:v>
       </x:c>
       <x:c r="D104" s="4" t="s">
+        <x:v>113</x:v>
+      </x:c>
+      <x:c r="E104" s="4" t="s">
         <x:v>114</x:v>
-      </x:c>
-      <x:c r="E104" s="4" t="s">
-        <x:v>115</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="15" hidden="0">
       <x:c r="A105" s="4" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B105" s="4" t="s">
-        <x:v>185</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="C105" s="5" t="n">
         <x:v>2.6E-005</x:v>
       </x:c>
       <x:c r="D105" s="4" t="s">
-        <x:v>114</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="E105" s="4" t="s">
-        <x:v>117</x:v>
+        <x:v>116</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="15" hidden="0">
       <x:c r="A106" s="4" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B106" s="4" t="s">
-        <x:v>186</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="C106" s="5" t="n">
         <x:v>0.00579</x:v>
       </x:c>
       <x:c r="D106" s="4" t="s">
-        <x:v>96</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="E106" s="4" t="s">
-        <x:v>119</x:v>
+        <x:v>118</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="15" hidden="0">
       <x:c r="A107" s="4" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B107" s="4" t="s">
-        <x:v>187</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="C107" s="5" t="n">
         <x:v>46.25</x:v>
       </x:c>
       <x:c r="D107" s="4" t="s">
-        <x:v>85</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="E107" s="4" t="s">
-        <x:v>121</x:v>
+        <x:v>120</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="15" hidden="0">
       <x:c r="A108" s="4" t="s">
+        <x:v>187</x:v>
+      </x:c>
+      <x:c r="B108" s="4" t="s">
         <x:v>188</x:v>
-      </x:c>
-      <x:c r="B108" s="4" t="s">
-        <x:v>189</x:v>
       </x:c>
       <x:c r="C108" s="5" t="n">
         <x:v>0.85</x:v>
@@ -3231,15 +3363,15 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="E108" s="4" t="s">
-        <x:v>190</x:v>
+        <x:v>189</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="15" hidden="0">
       <x:c r="A109" s="4" t="s">
-        <x:v>188</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="B109" s="4" t="s">
-        <x:v>191</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="C109" s="5" t="n">
         <x:v>0</x:v>
@@ -3248,15 +3380,15 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="E109" s="4" t="s">
-        <x:v>192</x:v>
+        <x:v>191</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="15" hidden="0">
       <x:c r="A110" s="4" t="s">
-        <x:v>188</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="B110" s="4" t="s">
-        <x:v>193</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="C110" s="5" t="n">
         <x:v>0.7</x:v>
@@ -3265,15 +3397,15 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="E110" s="4" t="s">
-        <x:v>194</x:v>
+        <x:v>193</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="15" hidden="0">
       <x:c r="A111" s="4" t="s">
-        <x:v>188</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="B111" s="4" t="s">
-        <x:v>195</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="C111" s="5" t="n">
         <x:v>0.7</x:v>
@@ -3282,83 +3414,83 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="E111" s="4" t="s">
-        <x:v>196</x:v>
+        <x:v>195</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="15" hidden="0">
       <x:c r="A112" s="4" t="s">
-        <x:v>188</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="B112" s="4" t="s">
-        <x:v>197</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="C112" s="5" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="D112" s="4" t="s">
+        <x:v>197</x:v>
+      </x:c>
+      <x:c r="E112" s="4" t="s">
         <x:v>198</x:v>
-      </x:c>
-      <x:c r="E112" s="4" t="s">
-        <x:v>199</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="15" hidden="0">
       <x:c r="A113" s="4" t="s">
-        <x:v>188</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="B113" s="4" t="s">
-        <x:v>200</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="C113" s="5" t="n">
         <x:v>12</x:v>
       </x:c>
       <x:c r="D113" s="4" t="s">
-        <x:v>198</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="E113" s="4" t="s">
-        <x:v>201</x:v>
+        <x:v>200</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="15" hidden="0">
       <x:c r="A114" s="4" t="s">
-        <x:v>188</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="B114" s="4" t="s">
-        <x:v>202</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="C114" s="5" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="D114" s="4" t="s">
+        <x:v>202</x:v>
+      </x:c>
+      <x:c r="E114" s="4" t="s">
         <x:v>203</x:v>
-      </x:c>
-      <x:c r="E114" s="4" t="s">
-        <x:v>204</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="15" hidden="0">
       <x:c r="A115" s="4" t="s">
-        <x:v>188</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="B115" s="4" t="s">
-        <x:v>205</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="C115" s="5" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="D115" s="4" t="s">
+        <x:v>205</x:v>
+      </x:c>
+      <x:c r="E115" s="4" t="s">
         <x:v>206</x:v>
-      </x:c>
-      <x:c r="E115" s="4" t="s">
-        <x:v>207</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="15" hidden="0">
       <x:c r="A116" s="4" t="s">
-        <x:v>188</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="B116" s="4" t="s">
-        <x:v>208</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="C116" s="5" t="n">
         <x:v>56</x:v>
@@ -3367,32 +3499,32 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="E116" s="4" t="s">
-        <x:v>209</x:v>
+        <x:v>208</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="15" hidden="0">
       <x:c r="A117" s="4" t="s">
-        <x:v>188</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="B117" s="4" t="s">
-        <x:v>210</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="C117" s="5" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D117" s="4" t="s">
-        <x:v>198</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="E117" s="4" t="s">
-        <x:v>211</x:v>
+        <x:v>210</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="15" hidden="0">
       <x:c r="A118" s="6" t="s">
-        <x:v>188</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="B118" s="6" t="s">
-        <x:v>212</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="C118" s="1" t="n">
         <x:v>0.7</x:v>
@@ -3401,15 +3533,15 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="E118" s="6" t="s">
-        <x:v>213</x:v>
+        <x:v>212</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="15" hidden="0">
       <x:c r="A119" s="6" t="s">
-        <x:v>188</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="B119" s="6" t="s">
-        <x:v>214</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="C119" s="1" t="n">
         <x:v>0.05</x:v>
@@ -3418,15 +3550,15 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="E119" s="6" t="s">
-        <x:v>215</x:v>
+        <x:v>214</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="15" hidden="0">
       <x:c r="A120" s="6" t="s">
-        <x:v>188</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="B120" s="6" t="s">
-        <x:v>216</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="C120" s="1" t="n">
         <x:v>-0.05</x:v>
@@ -3435,15 +3567,15 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="E120" s="6" t="s">
-        <x:v>217</x:v>
+        <x:v>216</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="15" hidden="0">
       <x:c r="A121" s="6" t="s">
-        <x:v>188</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="B121" s="6" t="s">
-        <x:v>218</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="C121" s="1" t="n">
         <x:v>0</x:v>
@@ -3452,15 +3584,15 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="E121" s="6" t="s">
-        <x:v>219</x:v>
+        <x:v>218</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="15" hidden="0">
       <x:c r="A122" s="6" t="s">
-        <x:v>188</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="B122" s="6" t="s">
-        <x:v>220</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="C122" s="1" t="n">
         <x:v>0</x:v>
@@ -3469,15 +3601,15 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="E122" s="6" t="s">
-        <x:v>221</x:v>
+        <x:v>220</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="15" hidden="0">
       <x:c r="A123" s="4" t="s">
+        <x:v>221</x:v>
+      </x:c>
+      <x:c r="B123" s="4" t="s">
         <x:v>222</x:v>
-      </x:c>
-      <x:c r="B123" s="4" t="s">
-        <x:v>223</x:v>
       </x:c>
       <x:c r="C123" s="5" t="n">
         <x:v>0.95</x:v>
@@ -3486,15 +3618,15 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="E123" s="4" t="s">
-        <x:v>224</x:v>
+        <x:v>223</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="15" hidden="0">
       <x:c r="A124" s="4" t="s">
-        <x:v>222</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="B124" s="4" t="s">
-        <x:v>225</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="C124" s="5" t="n">
         <x:v>33.5</x:v>
@@ -3503,134 +3635,134 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="E124" s="4" t="s">
-        <x:v>226</x:v>
+        <x:v>225</x:v>
       </x:c>
     </x:row>
     <x:row r="125" ht="15" hidden="0">
       <x:c r="A125" s="4" t="s">
-        <x:v>222</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="B125" s="4" t="s">
-        <x:v>227</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="C125" s="5" t="n">
         <x:v>0.01</x:v>
       </x:c>
       <x:c r="D125" s="4" t="s">
+        <x:v>227</x:v>
+      </x:c>
+      <x:c r="E125" s="4" t="s">
         <x:v>228</x:v>
-      </x:c>
-      <x:c r="E125" s="4" t="s">
-        <x:v>229</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="15" hidden="0">
       <x:c r="A126" s="4" t="s">
-        <x:v>222</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="B126" s="4" t="s">
-        <x:v>230</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="C126" s="5" t="n">
         <x:v>0.02</x:v>
       </x:c>
       <x:c r="D126" s="4" t="s">
-        <x:v>228</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="E126" s="4" t="s">
-        <x:v>231</x:v>
+        <x:v>230</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="15" hidden="0">
       <x:c r="A127" s="4" t="s">
-        <x:v>222</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="B127" s="4" t="s">
-        <x:v>232</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="C127" s="5" t="n">
         <x:v>7.9E-018</x:v>
       </x:c>
       <x:c r="D127" s="4" t="s">
+        <x:v>232</x:v>
+      </x:c>
+      <x:c r="E127" s="4" t="s">
         <x:v>233</x:v>
-      </x:c>
-      <x:c r="E127" s="4" t="s">
-        <x:v>234</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="15" hidden="0">
       <x:c r="A128" s="4" t="s">
-        <x:v>222</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="B128" s="4" t="s">
-        <x:v>235</x:v>
+        <x:v>234</x:v>
       </x:c>
       <x:c r="C128" s="5" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="D128" s="4" t="s">
+        <x:v>235</x:v>
+      </x:c>
+      <x:c r="E128" s="4" t="s">
         <x:v>236</x:v>
-      </x:c>
-      <x:c r="E128" s="4" t="s">
-        <x:v>237</x:v>
       </x:c>
     </x:row>
     <x:row r="129" ht="15" hidden="0">
       <x:c r="A129" s="4" t="s">
-        <x:v>222</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="B129" s="4" t="s">
-        <x:v>238</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="C129" s="5" t="n">
         <x:v>1E-007</x:v>
       </x:c>
       <x:c r="D129" s="4" t="s">
+        <x:v>238</x:v>
+      </x:c>
+      <x:c r="E129" s="4" t="s">
         <x:v>239</x:v>
-      </x:c>
-      <x:c r="E129" s="4" t="s">
-        <x:v>240</x:v>
       </x:c>
     </x:row>
     <x:row r="130" ht="15" hidden="0">
       <x:c r="A130" s="4" t="s">
-        <x:v>222</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="B130" s="4" t="s">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="C130" s="5" t="s">
         <x:v>241</x:v>
-      </x:c>
-      <x:c r="C130" s="5" t="s">
-        <x:v>242</x:v>
       </x:c>
       <x:c r="D130" s="4" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="E130" s="4" t="s">
-        <x:v>243</x:v>
+        <x:v>242</x:v>
       </x:c>
     </x:row>
     <x:row r="131" ht="15" hidden="0">
       <x:c r="A131" s="4" t="s">
+        <x:v>243</x:v>
+      </x:c>
+      <x:c r="B131" s="4" t="s">
         <x:v>244</x:v>
-      </x:c>
-      <x:c r="B131" s="4" t="s">
-        <x:v>245</x:v>
       </x:c>
       <x:c r="C131" s="5" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="D131" s="4" t="s">
+        <x:v>245</x:v>
+      </x:c>
+      <x:c r="E131" s="4" t="s">
         <x:v>246</x:v>
-      </x:c>
-      <x:c r="E131" s="4" t="s">
-        <x:v>247</x:v>
       </x:c>
     </x:row>
     <x:row r="132" ht="15" hidden="0">
       <x:c r="A132" s="4" t="s">
-        <x:v>244</x:v>
+        <x:v>243</x:v>
       </x:c>
       <x:c r="B132" s="4" t="s">
-        <x:v>248</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="C132" s="5" t="n">
         <x:v>2E-005</x:v>
@@ -3639,30 +3771,30 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="E132" s="4" t="s">
-        <x:v>249</x:v>
+        <x:v>248</x:v>
       </x:c>
     </x:row>
     <x:row r="133" ht="15" hidden="0">
       <x:c r="A133" s="4" t="s">
+        <x:v>249</x:v>
+      </x:c>
+      <x:c r="B133" s="4" t="s">
         <x:v>250</x:v>
-      </x:c>
-      <x:c r="B133" s="4" t="s">
-        <x:v>251</x:v>
       </x:c>
       <x:c r="C133" s="5"/>
       <x:c r="D133" s="4" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="E133" s="4" t="s">
-        <x:v>252</x:v>
+        <x:v>251</x:v>
       </x:c>
     </x:row>
     <x:row r="134" ht="15" hidden="0">
       <x:c r="A134" s="4" t="s">
-        <x:v>250</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="B134" s="4" t="s">
-        <x:v>253</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="C134" s="5" t="n">
         <x:v>0.001</x:v>
@@ -3671,47 +3803,47 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="E134" s="4" t="s">
-        <x:v>254</x:v>
+        <x:v>253</x:v>
       </x:c>
     </x:row>
     <x:row r="135" ht="15" hidden="0">
       <x:c r="A135" s="4" t="s">
-        <x:v>250</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="B135" s="4" t="s">
-        <x:v>255</x:v>
+        <x:v>254</x:v>
       </x:c>
       <x:c r="C135" s="5" t="n">
         <x:v>1E-005</x:v>
       </x:c>
       <x:c r="D135" s="4" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="E135" s="4" t="s">
-        <x:v>254</x:v>
+        <x:v>253</x:v>
       </x:c>
     </x:row>
     <x:row r="136" ht="15" hidden="0">
       <x:c r="A136" s="4" t="s">
-        <x:v>250</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="B136" s="4" t="s">
-        <x:v>256</x:v>
+        <x:v>255</x:v>
       </x:c>
       <x:c r="C136" s="5"/>
       <x:c r="D136" s="4" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="E136" s="4" t="s">
-        <x:v>252</x:v>
+        <x:v>251</x:v>
       </x:c>
     </x:row>
     <x:row r="137" ht="15" hidden="0">
       <x:c r="A137" s="4" t="s">
-        <x:v>250</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="B137" s="4" t="s">
-        <x:v>257</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="C137" s="5" t="n">
         <x:v>0.001</x:v>
@@ -3720,41 +3852,41 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="E137" s="4" t="s">
-        <x:v>254</x:v>
+        <x:v>253</x:v>
       </x:c>
     </x:row>
     <x:row r="138" ht="15" hidden="0">
       <x:c r="A138" s="4" t="s">
-        <x:v>250</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="B138" s="4" t="s">
-        <x:v>258</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="C138" s="5" t="n">
         <x:v>0.99999</x:v>
       </x:c>
       <x:c r="D138" s="4" t="s">
-        <x:v>239</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="E138" s="4" t="s">
-        <x:v>259</x:v>
+        <x:v>258</x:v>
       </x:c>
     </x:row>
     <x:row r="139" ht="15" hidden="0">
       <x:c r="A139" s="4" t="s">
-        <x:v>250</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="B139" s="4" t="s">
-        <x:v>260</x:v>
+        <x:v>259</x:v>
       </x:c>
       <x:c r="C139" s="5" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="D139" s="4" t="s">
+        <x:v>260</x:v>
+      </x:c>
+      <x:c r="E139" s="4" t="s">
         <x:v>261</x:v>
-      </x:c>
-      <x:c r="E139" s="4" t="s">
-        <x:v>262</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3778,7 +3910,7 @@
   <x:sheetData>
     <x:row r="1" ht="17.350000381469727" hidden="0">
       <x:c r="A1" s="2" t="s">
-        <x:v>263</x:v>
+        <x:v>262</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -3790,10 +3922,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="3" t="s">
+        <x:v>263</x:v>
+      </x:c>
+      <x:c r="C3" s="3" t="s">
         <x:v>264</x:v>
-      </x:c>
-      <x:c r="C3" s="3" t="s">
-        <x:v>265</x:v>
       </x:c>
       <x:c r="D3" s="3" t="s">
         <x:v>4</x:v>
@@ -3811,13 +3943,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C4" s="5" t="s">
-        <x:v>266</x:v>
+        <x:v>265</x:v>
       </x:c>
       <x:c r="D4" s="4" t="s">
         <x:v>28</x:v>
       </x:c>
       <x:c r="E4" s="4" t="s">
-        <x:v>267</x:v>
+        <x:v>266</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0">
@@ -3829,13 +3961,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C5" s="5" t="s">
-        <x:v>268</x:v>
+        <x:v>267</x:v>
       </x:c>
       <x:c r="D5" s="4" t="s">
         <x:v>28</x:v>
       </x:c>
       <x:c r="E5" s="4" t="s">
-        <x:v>269</x:v>
+        <x:v>268</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0">
@@ -3847,13 +3979,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C6" s="5" t="s">
-        <x:v>270</x:v>
+        <x:v>269</x:v>
       </x:c>
       <x:c r="D6" s="4" t="s">
         <x:v>28</x:v>
       </x:c>
       <x:c r="E6" s="4" t="s">
-        <x:v>271</x:v>
+        <x:v>270</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0">
@@ -3865,13 +3997,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C7" s="5" t="s">
-        <x:v>272</x:v>
+        <x:v>271</x:v>
       </x:c>
       <x:c r="D7" s="4" t="s">
         <x:v>47</x:v>
       </x:c>
       <x:c r="E7" s="4" t="s">
-        <x:v>273</x:v>
+        <x:v>272</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0">
@@ -3883,18 +4015,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C8" s="5" t="s">
-        <x:v>274</x:v>
+        <x:v>273</x:v>
       </x:c>
       <x:c r="D8" s="4" t="s">
         <x:v>47</x:v>
       </x:c>
       <x:c r="E8" s="4" t="s">
-        <x:v>275</x:v>
+        <x:v>274</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0">
       <x:c r="A9" s="4" t="s">
-        <x:v>276</x:v>
+        <x:v>275</x:v>
       </x:c>
       <x:c r="B9" s="4" t="b">
         <x:f aca="0">TRUE()</x:f>
@@ -3904,15 +4036,15 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="D9" s="4" t="s">
+        <x:v>276</x:v>
+      </x:c>
+      <x:c r="E9" s="4" t="s">
         <x:v>277</x:v>
-      </x:c>
-      <x:c r="E9" s="4" t="s">
-        <x:v>278</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0">
       <x:c r="A10" s="4" t="s">
-        <x:v>279</x:v>
+        <x:v>278</x:v>
       </x:c>
       <x:c r="B10" s="4" t="b">
         <x:f aca="0">TRUE()</x:f>
@@ -3923,15 +4055,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="D10" s="4" t="s">
-        <x:v>101</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="E10" s="4" t="s">
-        <x:v>280</x:v>
+        <x:v>279</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0">
       <x:c r="A11" s="4" t="s">
-        <x:v>281</x:v>
+        <x:v>280</x:v>
       </x:c>
       <x:c r="B11" s="4" t="b">
         <x:f aca="0">TRUE()</x:f>
@@ -3942,10 +4074,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D11" s="4" t="s">
-        <x:v>101</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="E11" s="4" t="s">
-        <x:v>282</x:v>
+        <x:v>281</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3972,7 +4104,7 @@
   <x:sheetData>
     <x:row r="1" ht="17.350000381469727" hidden="0">
       <x:c r="A1" s="2" t="s">
-        <x:v>283</x:v>
+        <x:v>282</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -3985,28 +4117,28 @@
     </x:row>
     <x:row r="3" ht="15" hidden="0">
       <x:c r="A3" s="3" t="s">
+        <x:v>283</x:v>
+      </x:c>
+      <x:c r="B3" s="3" t="s">
         <x:v>284</x:v>
       </x:c>
-      <x:c r="B3" s="3" t="s">
+      <x:c r="C3" s="3" t="s">
         <x:v>285</x:v>
       </x:c>
-      <x:c r="C3" s="3" t="s">
+      <x:c r="D3" s="3" t="s">
         <x:v>286</x:v>
       </x:c>
-      <x:c r="D3" s="3" t="s">
+      <x:c r="E3" s="3" t="s">
         <x:v>287</x:v>
       </x:c>
-      <x:c r="E3" s="3" t="s">
+      <x:c r="F3" s="3" t="s">
         <x:v>288</x:v>
       </x:c>
-      <x:c r="F3" s="3" t="s">
+      <x:c r="G3" s="3" t="s">
         <x:v>289</x:v>
       </x:c>
-      <x:c r="G3" s="3" t="s">
+      <x:c r="H3" s="3" t="s">
         <x:v>290</x:v>
-      </x:c>
-      <x:c r="H3" s="3" t="s">
-        <x:v>291</x:v>
       </x:c>
       <x:c r="I3" s="3" t="s">
         <x:v>5</x:v>
@@ -4014,16 +4146,16 @@
     </x:row>
     <x:row r="4" ht="15" hidden="0">
       <x:c r="A4" s="4" t="s">
+        <x:v>291</x:v>
+      </x:c>
+      <x:c r="B4" s="4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C4" s="5" t="s">
         <x:v>292</x:v>
       </x:c>
-      <x:c r="B4" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C4" s="5" t="s">
+      <x:c r="D4" s="4" t="s">
         <x:v>293</x:v>
-      </x:c>
-      <x:c r="D4" s="4" t="s">
-        <x:v>294</x:v>
       </x:c>
       <x:c r="E4" s="4" t="n">
         <x:v>46.25</x:v>
@@ -4039,21 +4171,21 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I4" s="4" t="s">
-        <x:v>295</x:v>
+        <x:v>294</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0">
       <x:c r="A5" s="4" t="s">
-        <x:v>296</x:v>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="B5" s="4" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C5" s="5" t="s">
-        <x:v>297</x:v>
+        <x:v>296</x:v>
       </x:c>
       <x:c r="D5" s="4" t="s">
-        <x:v>294</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="E5" s="4" t="n">
         <x:v>46.25</x:v>
@@ -4069,21 +4201,21 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I5" s="4" t="s">
-        <x:v>298</x:v>
+        <x:v>297</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0">
       <x:c r="A6" s="4" t="s">
-        <x:v>296</x:v>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="B6" s="4" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="C6" s="5" t="s">
-        <x:v>299</x:v>
+        <x:v>298</x:v>
       </x:c>
       <x:c r="D6" s="4" t="s">
-        <x:v>294</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="E6" s="4" t="n">
         <x:v>46.25</x:v>
@@ -4099,21 +4231,21 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I6" s="4" t="s">
-        <x:v>300</x:v>
+        <x:v>299</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0">
       <x:c r="A7" s="4" t="s">
-        <x:v>296</x:v>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="B7" s="4" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="C7" s="5" t="s">
-        <x:v>301</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="D7" s="4" t="s">
-        <x:v>294</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="E7" s="4" t="n">
         <x:v>46.25</x:v>
@@ -4129,21 +4261,21 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I7" s="4" t="s">
-        <x:v>302</x:v>
+        <x:v>301</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0">
       <x:c r="A8" s="4" t="s">
-        <x:v>296</x:v>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="B8" s="4" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C8" s="5" t="s">
-        <x:v>303</x:v>
+        <x:v>302</x:v>
       </x:c>
       <x:c r="D8" s="4" t="s">
-        <x:v>294</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="E8" s="4" t="n">
         <x:v>46.25</x:v>
@@ -4159,21 +4291,21 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I8" s="4" t="s">
-        <x:v>304</x:v>
+        <x:v>303</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0">
       <x:c r="A9" s="4" t="s">
-        <x:v>296</x:v>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="B9" s="4" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C9" s="5" t="s">
-        <x:v>305</x:v>
+        <x:v>304</x:v>
       </x:c>
       <x:c r="D9" s="4" t="s">
-        <x:v>294</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="E9" s="4" t="n">
         <x:v>46.25</x:v>
@@ -4189,21 +4321,21 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I9" s="4" t="s">
-        <x:v>306</x:v>
+        <x:v>305</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0">
       <x:c r="A10" s="4" t="s">
-        <x:v>296</x:v>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="B10" s="4" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="C10" s="5" t="s">
-        <x:v>307</x:v>
+        <x:v>306</x:v>
       </x:c>
       <x:c r="D10" s="4" t="s">
-        <x:v>294</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="E10" s="4" t="n">
         <x:v>46.25</x:v>
@@ -4219,21 +4351,21 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I10" s="4" t="s">
-        <x:v>308</x:v>
+        <x:v>307</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0">
       <x:c r="A11" s="4" t="s">
-        <x:v>309</x:v>
+        <x:v>308</x:v>
       </x:c>
       <x:c r="B11" s="4" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C11" s="5" t="s">
-        <x:v>310</x:v>
+        <x:v>309</x:v>
       </x:c>
       <x:c r="D11" s="4" t="s">
-        <x:v>294</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="E11" s="4" t="n">
         <x:v>46.25</x:v>
@@ -4249,21 +4381,21 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I11" s="4" t="s">
-        <x:v>311</x:v>
+        <x:v>310</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0">
       <x:c r="A12" s="4" t="s">
-        <x:v>309</x:v>
+        <x:v>308</x:v>
       </x:c>
       <x:c r="B12" s="4" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="C12" s="5" t="s">
-        <x:v>312</x:v>
+        <x:v>311</x:v>
       </x:c>
       <x:c r="D12" s="4" t="s">
-        <x:v>294</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="E12" s="4" t="n">
         <x:v>46.25</x:v>
@@ -4279,21 +4411,21 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I12" s="4" t="s">
-        <x:v>313</x:v>
+        <x:v>312</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0">
       <x:c r="A13" s="4" t="s">
-        <x:v>309</x:v>
+        <x:v>308</x:v>
       </x:c>
       <x:c r="B13" s="4" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="C13" s="5" t="s">
-        <x:v>314</x:v>
+        <x:v>313</x:v>
       </x:c>
       <x:c r="D13" s="4" t="s">
-        <x:v>294</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="E13" s="4" t="n">
         <x:v>46.25</x:v>
@@ -4309,21 +4441,21 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I13" s="4" t="s">
-        <x:v>315</x:v>
+        <x:v>314</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0">
       <x:c r="A14" s="4" t="s">
-        <x:v>309</x:v>
+        <x:v>308</x:v>
       </x:c>
       <x:c r="B14" s="4" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C14" s="5" t="s">
-        <x:v>316</x:v>
+        <x:v>315</x:v>
       </x:c>
       <x:c r="D14" s="4" t="s">
-        <x:v>294</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="E14" s="4" t="n">
         <x:v>46.25</x:v>
@@ -4339,21 +4471,21 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I14" s="4" t="s">
-        <x:v>317</x:v>
+        <x:v>316</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0">
       <x:c r="A15" s="4" t="s">
-        <x:v>309</x:v>
+        <x:v>308</x:v>
       </x:c>
       <x:c r="B15" s="4" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C15" s="5" t="s">
-        <x:v>318</x:v>
+        <x:v>317</x:v>
       </x:c>
       <x:c r="D15" s="4" t="s">
-        <x:v>294</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="E15" s="4" t="n">
         <x:v>46.25</x:v>
@@ -4369,7 +4501,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I15" s="4" t="s">
-        <x:v>319</x:v>
+        <x:v>318</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4384,25 +4516,25 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="13.029999732971191" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="20.950000762939453" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="15.119999885559082" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="5.840000152587891" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="46.5099983215332" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="13.029999732971191" style="7" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20.950000762939453" style="7" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="15.119999885559082" style="7" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="5.840000152587891" style="7" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="46.5099983215332" style="7" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0">
-      <x:c r="A1" s="7" t="s">
-        <x:v>320</x:v>
-      </x:c>
-      <x:c r="B1" s="7"/>
-      <x:c r="C1" s="7"/>
-      <x:c r="D1" s="7"/>
-      <x:c r="E1" s="7"/>
+      <x:c r="A1" s="8" t="s">
+        <x:v>319</x:v>
+      </x:c>
+      <x:c r="B1" s="8"/>
+      <x:c r="C1" s="8"/>
+      <x:c r="D1" s="8"/>
+      <x:c r="E1" s="8"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0">
       <x:c r="A3" s="6" t="s">
-        <x:v>321</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="B3" s="6" t="s">
         <x:v>2</x:v>
@@ -4418,343 +4550,343 @@
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0">
-      <x:c r="A4" s="6" t="str">
-        <x:v>single_run</x:v>
-      </x:c>
-      <x:c r="B4" s="6" t="str">
-        <x:v>target</x:v>
-      </x:c>
-      <x:c r="C4" s="6" t="str">
-        <x:v>dfe</x:v>
-      </x:c>
-      <x:c r="D4" s="6" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="E4" s="6" t="str">
-        <x:v>Full single-run target.</x:v>
+      <x:c r="A4" s="6" t="s">
+        <x:v>321</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="s">
+        <x:v>322</x:v>
+      </x:c>
+      <x:c r="C4" s="6" t="s">
+        <x:v>323</x:v>
+      </x:c>
+      <x:c r="D4" s="6" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E4" s="6" t="s">
+        <x:v>324</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0">
-      <x:c r="A5" s="6" t="str">
-        <x:v>single_run</x:v>
-      </x:c>
-      <x:c r="B5" s="6" t="str">
-        <x:v>pre_dte_pmf_method</x:v>
-      </x:c>
-      <x:c r="C5" s="6" t="str">
-        <x:v>pmf_exact</x:v>
-      </x:c>
-      <x:c r="D5" s="6" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="E5" s="6" t="str">
-        <x:v>Pre-DTE ADC PMF method for V_qc.</x:v>
+      <x:c r="A5" s="6" t="s">
+        <x:v>321</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="s">
+        <x:v>325</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="s">
+        <x:v>241</x:v>
+      </x:c>
+      <x:c r="D5" s="6" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E5" s="6" t="s">
+        <x:v>326</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0">
-      <x:c r="A6" s="6" t="str">
-        <x:v>single_run</x:v>
-      </x:c>
-      <x:c r="B6" s="6" t="str">
-        <x:v>pmf_grid_quality</x:v>
-      </x:c>
-      <x:c r="C6" s="6" t="str">
-        <x:v>fine</x:v>
-      </x:c>
-      <x:c r="D6" s="6" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="E6" s="6" t="str">
-        <x:v>PMF amplitude-grid quality.</x:v>
+      <x:c r="A6" s="6" t="s">
+        <x:v>321</x:v>
+      </x:c>
+      <x:c r="B6" s="6" t="s">
+        <x:v>327</x:v>
+      </x:c>
+      <x:c r="C6" s="6" t="s">
+        <x:v>328</x:v>
+      </x:c>
+      <x:c r="D6" s="6" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E6" s="6" t="s">
+        <x:v>329</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0">
-      <x:c r="A7" s="6" t="str">
-        <x:v>single_run</x:v>
-      </x:c>
-      <x:c r="B7" s="6" t="str">
-        <x:v>floating_mode</x:v>
-      </x:c>
-      <x:c r="C7" s="6" t="str">
-        <x:v>simplified</x:v>
-      </x:c>
-      <x:c r="D7" s="6" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="E7" s="6" t="str">
-        <x:v>FFE floating-group selection.</x:v>
+      <x:c r="A7" s="6" t="s">
+        <x:v>321</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="s">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="C7" s="6" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="D7" s="6" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E7" s="6" t="s">
+        <x:v>332</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0">
-      <x:c r="A8" s="6" t="str">
-        <x:v>single_run</x:v>
-      </x:c>
-      <x:c r="B8" s="6" t="str">
-        <x:v>pos_sweep_method</x:v>
-      </x:c>
-      <x:c r="C8" s="6" t="str">
-        <x:v>each_phase</x:v>
-      </x:c>
-      <x:c r="D8" s="6" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="E8" s="6" t="str">
-        <x:v>Sampling-phase sweep strategy.</x:v>
+      <x:c r="A8" s="6" t="s">
+        <x:v>321</x:v>
+      </x:c>
+      <x:c r="B8" s="6" t="s">
+        <x:v>333</x:v>
+      </x:c>
+      <x:c r="C8" s="6" t="s">
+        <x:v>334</x:v>
+      </x:c>
+      <x:c r="D8" s="6" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E8" s="6" t="s">
+        <x:v>335</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0">
-      <x:c r="A9" s="6" t="str">
-        <x:v>single_run</x:v>
-      </x:c>
-      <x:c r="B9" s="6" t="str">
-        <x:v>pos_coarse_stride</x:v>
+      <x:c r="A9" s="6" t="s">
+        <x:v>321</x:v>
+      </x:c>
+      <x:c r="B9" s="6" t="s">
+        <x:v>336</x:v>
       </x:c>
       <x:c r="C9" s="6" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="D9" s="6" t="str">
-        <x:v>phase index</x:v>
-      </x:c>
-      <x:c r="E9" s="6" t="str">
-        <x:v>Coarse phase stride; used only by coarse_fine.</x:v>
+      <x:c r="D9" s="6" t="s">
+        <x:v>337</x:v>
+      </x:c>
+      <x:c r="E9" s="6" t="s">
+        <x:v>338</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0">
-      <x:c r="A10" s="6" t="str">
-        <x:v>search_sweep</x:v>
-      </x:c>
-      <x:c r="B10" s="6" t="str">
-        <x:v>target</x:v>
-      </x:c>
-      <x:c r="C10" s="6" t="str">
-        <x:v>mse</x:v>
-      </x:c>
-      <x:c r="D10" s="6" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="E10" s="6" t="str">
-        <x:v>Partial-search candidate evaluation target.</x:v>
+      <x:c r="A10" s="6" t="s">
+        <x:v>339</x:v>
+      </x:c>
+      <x:c r="B10" s="6" t="s">
+        <x:v>322</x:v>
+      </x:c>
+      <x:c r="C10" s="6" t="s">
+        <x:v>340</x:v>
+      </x:c>
+      <x:c r="D10" s="6" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E10" s="6" t="s">
+        <x:v>341</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0">
-      <x:c r="A11" s="6" t="str">
-        <x:v>search_sweep</x:v>
-      </x:c>
-      <x:c r="B11" s="6" t="str">
-        <x:v>pre_dte_pmf_method</x:v>
-      </x:c>
-      <x:c r="C11" s="6" t="str">
-        <x:v>gaussian_approx</x:v>
-      </x:c>
-      <x:c r="D11" s="6" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="E11" s="6" t="str">
-        <x:v>Pre-DTE ADC PMF method for V_qc.</x:v>
+      <x:c r="A11" s="6" t="s">
+        <x:v>339</x:v>
+      </x:c>
+      <x:c r="B11" s="6" t="s">
+        <x:v>325</x:v>
+      </x:c>
+      <x:c r="C11" s="6" t="s">
+        <x:v>241</x:v>
+      </x:c>
+      <x:c r="D11" s="6" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E11" s="6" t="s">
+        <x:v>326</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0">
-      <x:c r="A12" s="6" t="str">
-        <x:v>search_sweep</x:v>
-      </x:c>
-      <x:c r="B12" s="6" t="str">
-        <x:v>pmf_grid_quality</x:v>
-      </x:c>
-      <x:c r="C12" s="6" t="str">
-        <x:v>coarse</x:v>
-      </x:c>
-      <x:c r="D12" s="6" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="E12" s="6" t="str">
-        <x:v>PMF amplitude-grid quality.</x:v>
+      <x:c r="A12" s="6" t="s">
+        <x:v>339</x:v>
+      </x:c>
+      <x:c r="B12" s="6" t="s">
+        <x:v>327</x:v>
+      </x:c>
+      <x:c r="C12" s="6" t="s">
+        <x:v>328</x:v>
+      </x:c>
+      <x:c r="D12" s="6" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E12" s="6" t="s">
+        <x:v>329</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0">
-      <x:c r="A13" s="6" t="str">
-        <x:v>search_sweep</x:v>
-      </x:c>
-      <x:c r="B13" s="6" t="str">
-        <x:v>floating_mode</x:v>
-      </x:c>
-      <x:c r="C13" s="1" t="str">
-        <x:v>heuristic</x:v>
-      </x:c>
-      <x:c r="D13" s="6" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="E13" s="6" t="str">
-        <x:v>FFE floating-group selection.</x:v>
+      <x:c r="A13" s="6" t="s">
+        <x:v>339</x:v>
+      </x:c>
+      <x:c r="B13" s="6" t="s">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="C13" s="9" t="s">
+        <x:v>342</x:v>
+      </x:c>
+      <x:c r="D13" s="6" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E13" s="6" t="s">
+        <x:v>332</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0">
-      <x:c r="A14" s="6" t="str">
-        <x:v>search_sweep</x:v>
-      </x:c>
-      <x:c r="B14" s="6" t="str">
-        <x:v>pos_sweep_method</x:v>
-      </x:c>
-      <x:c r="C14" s="1" t="str">
-        <x:v>coarse_fine</x:v>
-      </x:c>
-      <x:c r="D14" s="6" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="E14" s="6" t="str">
-        <x:v>Sampling-phase sweep strategy.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" t="str">
-        <x:v>search_sweep</x:v>
-      </x:c>
-      <x:c r="B15" t="str">
-        <x:v>pos_coarse_stride</x:v>
-      </x:c>
-      <x:c r="C15" t="n">
+      <x:c r="A14" s="6" t="s">
+        <x:v>339</x:v>
+      </x:c>
+      <x:c r="B14" s="6" t="s">
+        <x:v>333</x:v>
+      </x:c>
+      <x:c r="C14" s="9" t="s">
+        <x:v>343</x:v>
+      </x:c>
+      <x:c r="D14" s="6" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E14" s="6" t="s">
+        <x:v>335</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0">
+      <x:c r="A15" s="10" t="s">
+        <x:v>339</x:v>
+      </x:c>
+      <x:c r="B15" s="10" t="s">
+        <x:v>336</x:v>
+      </x:c>
+      <x:c r="C15" s="10" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="D15" t="str">
-        <x:v>phase index</x:v>
-      </x:c>
-      <x:c r="E15" t="str">
-        <x:v>Coarse phase stride; used only by coarse_fine.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" t="str">
-        <x:v>search_final</x:v>
-      </x:c>
-      <x:c r="B16" t="str">
-        <x:v>target</x:v>
-      </x:c>
-      <x:c r="C16" t="str">
-        <x:v>dfe</x:v>
-      </x:c>
-      <x:c r="D16" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="E16" t="str">
-        <x:v>Top-K final evaluation target.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" t="str">
-        <x:v>search_final</x:v>
-      </x:c>
-      <x:c r="B17" t="str">
-        <x:v>pre_dte_pmf_method</x:v>
-      </x:c>
-      <x:c r="C17" t="str">
-        <x:v>gaussian_approx</x:v>
-      </x:c>
-      <x:c r="D17" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="E17" t="str">
-        <x:v>Pre-DTE ADC PMF method for V_qc.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" t="str">
-        <x:v>search_final</x:v>
-      </x:c>
-      <x:c r="B18" t="str">
-        <x:v>pmf_grid_quality</x:v>
-      </x:c>
-      <x:c r="C18" t="str">
-        <x:v>fine</x:v>
-      </x:c>
-      <x:c r="D18" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="E18" t="str">
-        <x:v>PMF amplitude-grid quality.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" t="str">
-        <x:v>search_final</x:v>
-      </x:c>
-      <x:c r="B19" t="str">
-        <x:v>floating_mode</x:v>
-      </x:c>
-      <x:c r="C19" t="str">
-        <x:v>heuristic</x:v>
-      </x:c>
-      <x:c r="D19" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="E19" t="str">
-        <x:v>FFE floating-group selection.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" t="str">
-        <x:v>search_final</x:v>
-      </x:c>
-      <x:c r="B20" t="str">
-        <x:v>pos_sweep_method</x:v>
-      </x:c>
-      <x:c r="C20" t="str">
-        <x:v>each_phase</x:v>
-      </x:c>
-      <x:c r="D20" t="str">
-        <x:v>text</x:v>
-      </x:c>
-      <x:c r="E20" t="str">
-        <x:v>Sampling-phase sweep strategy.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" t="str">
-        <x:v>search_final</x:v>
-      </x:c>
-      <x:c r="B21" t="str">
-        <x:v>pos_coarse_stride</x:v>
-      </x:c>
-      <x:c r="C21" t="n">
+      <x:c r="D15" s="10" t="s">
+        <x:v>337</x:v>
+      </x:c>
+      <x:c r="E15" s="10" t="s">
+        <x:v>338</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0">
+      <x:c r="A16" s="10" t="s">
+        <x:v>344</x:v>
+      </x:c>
+      <x:c r="B16" s="10" t="s">
+        <x:v>322</x:v>
+      </x:c>
+      <x:c r="C16" s="10" t="s">
+        <x:v>323</x:v>
+      </x:c>
+      <x:c r="D16" s="10" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E16" s="10" t="s">
+        <x:v>345</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0">
+      <x:c r="A17" s="10" t="s">
+        <x:v>344</x:v>
+      </x:c>
+      <x:c r="B17" s="10" t="s">
+        <x:v>325</x:v>
+      </x:c>
+      <x:c r="C17" s="10" t="s">
+        <x:v>241</x:v>
+      </x:c>
+      <x:c r="D17" s="10" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E17" s="10" t="s">
+        <x:v>326</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0">
+      <x:c r="A18" s="10" t="s">
+        <x:v>344</x:v>
+      </x:c>
+      <x:c r="B18" s="10" t="s">
+        <x:v>327</x:v>
+      </x:c>
+      <x:c r="C18" s="10" t="s">
+        <x:v>346</x:v>
+      </x:c>
+      <x:c r="D18" s="10" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E18" s="10" t="s">
+        <x:v>329</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0">
+      <x:c r="A19" s="10" t="s">
+        <x:v>344</x:v>
+      </x:c>
+      <x:c r="B19" s="10" t="s">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="C19" s="10" t="s">
+        <x:v>342</x:v>
+      </x:c>
+      <x:c r="D19" s="10" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E19" s="10" t="s">
+        <x:v>332</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="15" hidden="0">
+      <x:c r="A20" s="10" t="s">
+        <x:v>344</x:v>
+      </x:c>
+      <x:c r="B20" s="10" t="s">
+        <x:v>333</x:v>
+      </x:c>
+      <x:c r="C20" s="10" t="s">
+        <x:v>334</x:v>
+      </x:c>
+      <x:c r="D20" s="10" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E20" s="10" t="s">
+        <x:v>335</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0">
+      <x:c r="A21" s="10" t="s">
+        <x:v>344</x:v>
+      </x:c>
+      <x:c r="B21" s="10" t="s">
+        <x:v>336</x:v>
+      </x:c>
+      <x:c r="C21" s="10" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="D21" t="str">
-        <x:v>phase index</x:v>
-      </x:c>
-      <x:c r="E21" t="str">
-        <x:v>Coarse phase stride; used only by coarse_fine.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" t="str">
-        <x:v>search</x:v>
-      </x:c>
-      <x:c r="B22" t="str">
-        <x:v>group_size</x:v>
-      </x:c>
-      <x:c r="C22" t="n">
+      <x:c r="D21" s="10" t="s">
+        <x:v>337</x:v>
+      </x:c>
+      <x:c r="E21" s="10" t="s">
+        <x:v>338</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="15" hidden="0">
+      <x:c r="A22" s="10" t="s">
+        <x:v>347</x:v>
+      </x:c>
+      <x:c r="B22" s="10" t="s">
+        <x:v>348</x:v>
+      </x:c>
+      <x:c r="C22" s="7" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="D22" t="str">
-        <x:v>count</x:v>
-      </x:c>
-      <x:c r="E22" t="str">
-        <x:v>Manifest candidates per partial-search group.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" t="str">
-        <x:v>search</x:v>
-      </x:c>
-      <x:c r="B23" t="str">
-        <x:v>top_k</x:v>
-      </x:c>
-      <x:c r="C23" t="n">
+      <x:c r="D22" s="10" t="s">
+        <x:v>276</x:v>
+      </x:c>
+      <x:c r="E22" s="10" t="s">
+        <x:v>349</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="15" hidden="0">
+      <x:c r="A23" s="10" t="s">
+        <x:v>347</x:v>
+      </x:c>
+      <x:c r="B23" s="10" t="s">
+        <x:v>350</x:v>
+      </x:c>
+      <x:c r="C23" s="7" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="D23" t="str">
-        <x:v>count</x:v>
-      </x:c>
-      <x:c r="E23" t="str">
-        <x:v>Minimum-MSE candidates re-evaluated by search_final.</x:v>
+      <x:c r="D23" s="10" t="s">
+        <x:v>276</x:v>
+      </x:c>
+      <x:c r="E23" s="10" t="s">
+        <x:v>351</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4762,60 +4894,75 @@
     <x:mergeCell ref="A1:E1"/>
   </x:mergeCells>
   <x:dataValidations count="18">
-    <x:dataValidation type="list" errorStyle="stop" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C4">
+    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C4">
       <x:formula1>"mse,dfe,mlsd,full"</x:formula1>
+      <x:formula2>0</x:formula2>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C5">
+    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C5">
       <x:formula1>"gaussian_approx,pmf_exact"</x:formula1>
+      <x:formula2>0</x:formula2>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C6">
+    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C6">
       <x:formula1>"coarse,fine"</x:formula1>
+      <x:formula2>0</x:formula2>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C7">
+    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C7">
       <x:formula1>"heuristic,simplified,spec-defined"</x:formula1>
+      <x:formula2>0</x:formula2>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C8">
+    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C8">
       <x:formula1>"each_phase,coarse_fine"</x:formula1>
+      <x:formula2>0</x:formula2>
     </x:dataValidation>
     <x:dataValidation type="whole" errorStyle="stop" operator="between" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C9">
       <x:formula1>1</x:formula1>
       <x:formula2>32</x:formula2>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C10">
+    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C10">
       <x:formula1>"mse,dfe,mlsd,full"</x:formula1>
+      <x:formula2>0</x:formula2>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C11">
+    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C11">
       <x:formula1>"gaussian_approx,pmf_exact"</x:formula1>
+      <x:formula2>0</x:formula2>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C12">
+    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C12">
       <x:formula1>"coarse,fine"</x:formula1>
+      <x:formula2>0</x:formula2>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="C14">
+    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C14">
       <x:formula1>"each_phase,coarse_fine"</x:formula1>
+      <x:formula2>0</x:formula2>
     </x:dataValidation>
-    <x:dataValidation type="whole" operator="between" sqref="C15">
+    <x:dataValidation type="whole" errorStyle="stop" operator="between" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C15">
       <x:formula1>1</x:formula1>
       <x:formula2>32</x:formula2>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="C16">
+    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C16">
       <x:formula1>"mse,dfe,mlsd,full"</x:formula1>
+      <x:formula2>0</x:formula2>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="C17">
+    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C17">
       <x:formula1>"gaussian_approx,pmf_exact"</x:formula1>
+      <x:formula2>0</x:formula2>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="C13">
+    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C13">
       <x:formula1>"heuristic,simplified,spec-defined"</x:formula1>
+      <x:formula2>0</x:formula2>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="C18">
+    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C18">
       <x:formula1>"coarse,fine"</x:formula1>
+      <x:formula2>0</x:formula2>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="C19">
+    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C19">
       <x:formula1>"heuristic,simplified,spec-defined"</x:formula1>
+      <x:formula2>0</x:formula2>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="C20">
+    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C20">
       <x:formula1>"each_phase,coarse_fine"</x:formula1>
+      <x:formula2>0</x:formula2>
     </x:dataValidation>
-    <x:dataValidation type="whole" operator="between" sqref="C21">
+    <x:dataValidation type="whole" errorStyle="stop" operator="between" allowBlank="0" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="C21">
       <x:formula1>1</x:formula1>
       <x:formula2>32</x:formula2>
     </x:dataValidation>

</xml_diff>